<commit_message>
Move modelling choices into the dashboard with a live Fit tab
The workbook now holds only data (losses, exposure, contract + reporting
threshold, valuation year, loss inflation). Modelling threshold, splice,
frequency model, simulations, and loadings are live controls. Splitting
fit_models (fast) from price_models (Monte Carlo) lets the Fit tab show the
mean-excess plot, fitted vs empirical severity, and live parameters as the
thresholds change; pricing runs on demand. read_input makes the modelling
params optional; resolve_settings layers overrides over the workbook over
defaults. Adds mean_excess and tests; 70 passing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2BJg9kV48JX9NLTE3S1mv
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -50,49 +50,10 @@
     <t xml:space="preserve">0.03</t>
   </si>
   <si>
-    <t xml:space="preserve">modelling_threshold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">splice_threshold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frequency_model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">poisson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n_simulations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">200000</t>
-  </si>
-  <si>
     <t xml:space="preserve">valuation_year</t>
   </si>
   <si>
     <t xml:space="preserve">2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loading_ev</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loading_sd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">var_level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.99</t>
   </si>
   <si>
     <t xml:space="preserve">deductible</t>
@@ -744,63 +705,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -816,22 +721,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Move contract structure into the dashboard
Add a Structure tab with an add/remove layer editor (pure Shiny) and
drop the contract sheet from the input workbook. The dashboard now owns
the program, seeded from a built-in default_contract(); the headless
run_pricing path takes the same structure via a contract argument. The
unused reinstatement_cost field is removed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -9,13 +9,12 @@
     <sheet name="losses" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="exposure" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="parameters" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="contract" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -54,24 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deductible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cover</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n_reinstatements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reinstatement_cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aal</t>
   </si>
 </sst>
 </file>
@@ -712,95 +693,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="n">
-        <v>999</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>10</v>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>999</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4" t="n">
-        <v>999</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Make loss inflation per-year and scale frequency by exposure
Inflation is now a per-year rate in its own 'inflation' sheet (replacing the
single loss_inflation_pa); index_losses compounds the rates of the years after
a loss up to the valuation year. The Data step shows an exposure-and-inflation
by-year table and the full scrollable loss list.

Exposure now also drives the projected claim frequency: fit_models scales the
observed-period rate by the forward book relative to the average observed book
(exposure_frequency_factor + scale_frequency), so a growing book produces
proportionally more claims. With flat exposure the factor is 1, so existing
behaviour is unchanged.

A "To discuss" note records that the dashboard should explain to users how the
exposure inputs are used (on-levelling and frequency scaling).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="losses" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="exposure" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="parameters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="inflation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="parameters" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -31,6 +32,9 @@
     <t xml:space="preserve">exposure</t>
   </si>
   <si>
+    <t xml:space="preserve">inflation</t>
+  </si>
+  <si>
     <t xml:space="preserve">key</t>
   </si>
   <si>
@@ -41,12 +45,6 @@
   </si>
   <si>
     <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loss_inflation_pa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.03</t>
   </si>
   <si>
     <t xml:space="preserve">valuation_year</t>
@@ -659,34 +657,93 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
         <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Style input.xlsx with navy headers to match the dashboard
Generate the template with bold white-on-navy (#1B2A4A) headers, light
cell borders, a frozen header row, inflation shown as a percentage, and
thousands separators. Styling only affects display; read_input reads the
underlying values unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SQtr67nYmnTHmNYLHPkrr6
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -57,8 +57,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -66,16 +70,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B2A4A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -83,12 +103,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1B2A4A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1B2A4A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1B2A4A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1B2A4A"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDDE3EC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDDE3EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDDE3EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDDE3EC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -378,202 +435,207 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -587,60 +649,64 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>120</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>120</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>130</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>140</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>145</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>150</v>
       </c>
     </row>
@@ -654,60 +720,64 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="5" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="5" t="n">
         <v>0.025</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="5" t="n">
         <v>0.04</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="5" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="5" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -721,28 +791,32 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="24.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Show the two premium loadings as separate method cards
Wrap each loading on the Price step in its own titled card stating the
method name and the formula it drives, so the expected value and standard
deviation methods read as alternatives rather than two margins added
together. Update the info panel wording to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,68 +1,72 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pacoe\coding_projects\Paco's Pricing Pipeline\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB069D01-17CA-4E76-B1F6-EC516739DA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="losses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="exposure" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="inflation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="parameters" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="losses" sheetId="1" r:id="rId1"/>
+    <sheet name="exposure" sheetId="2" r:id="rId2"/>
+    <sheet name="inflation" sheetId="3" r:id="rId3"/>
+    <sheet name="parameters" sheetId="4" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t xml:space="preserve">year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">line_of_business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">exposure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">inflation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reporting_threshold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valuation_year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>loss</t>
+  </si>
+  <si>
+    <t>line_of_business</t>
+  </si>
+  <si>
+    <t>fire</t>
+  </si>
+  <si>
+    <t>exposure</t>
+  </si>
+  <si>
+    <t>inflation</t>
+  </si>
+  <si>
+    <t>key</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>reporting_threshold</t>
+  </si>
+  <si>
+    <t>valuation_year</t>
+  </si>
+  <si>
+    <t>2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -71,10 +75,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <b/>
     </font>
     <font>
       <sz val="11"/>
@@ -116,6 +120,7 @@
       <bottom style="thin">
         <color rgb="FF1B2A4A"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -130,27 +135,41 @@
       <bottom style="thin">
         <color rgb="FFDDE3EC"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -432,16 +451,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -452,209 +471,149 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>2021</v>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>6</v>
+      <c r="B2" s="6">
+        <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>2021</v>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>8</v>
+      <c r="B3" s="6">
+        <v>9.5</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>22</v>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>2023</v>
+      </c>
+      <c r="B4" s="6">
+        <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>7</v>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>2024</v>
+      </c>
+      <c r="B5" s="6">
+        <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>35</v>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>2024</v>
+      </c>
+      <c r="B6" s="6">
+        <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>9</v>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>2024</v>
+      </c>
+      <c r="B7" s="6">
+        <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>11</v>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B8" s="6">
+        <v>14</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>3</v>
-      </c>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -662,70 +621,70 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>2021</v>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="B2" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>2022</v>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="B3" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>2023</v>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="B4" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>2024</v>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="B5" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>2025</v>
       </c>
-      <c r="B6" s="3" t="n">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="B6" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>2026</v>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>150</v>
+      <c r="B7" s="3">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -733,70 +692,70 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>2021</v>
       </c>
-      <c r="B2" s="5" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="B2" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>2022</v>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="B3" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>2023</v>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>0.025</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="B4" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>2024</v>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="B5" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>2025</v>
       </c>
-      <c r="B6" s="5" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="B6" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>2026</v>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>0.035</v>
+      <c r="B7" s="5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -804,24 +763,24 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+      <c r="B3" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rename the parameters sheet to general inputs; add optional currency and units
Rename the workbook's parameters sheet to "general inputs" and add two optional
fields, currency and amount_units, that label every figure. They are surfaced so
they are not inert: the Data step lists them, a caption marks the Results
("Amounts are in EUR millions"), the structure and severity plots label their
money axes, and the downloaded workbook records them. A notes column in the
sheet marks each field required or optional; the reader ignores extra columns and
treats currency/units as optional. Updates the example template, input.xlsx,
tests (105 pass), the documentation and the Word copy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,29 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pacoe\coding_projects\Paco's Pricing Pipeline\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB069D01-17CA-4E76-B1F6-EC516739DA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2265" yWindow="2265" windowWidth="28800" windowHeight="15345" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="losses" sheetId="1" r:id="rId1"/>
-    <sheet name="exposure" sheetId="2" r:id="rId2"/>
-    <sheet name="inflation" sheetId="3" r:id="rId3"/>
-    <sheet name="parameters" sheetId="4" r:id="rId4"/>
+    <sheet name="losses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="exposure" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="inflation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="general inputs" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>year</t>
   </si>
@@ -56,6 +49,42 @@
   </si>
   <si>
     <t>2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valuation_year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required: the year losses are revalued to.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">currency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional: shown next to amounts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amount_units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">millions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional: shown next to amounts (e.g. millions, thousands).</t>
   </si>
 </sst>
 </file>
@@ -63,10 +92,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -75,10 +104,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <b/>
     </font>
     <font>
       <sz val="11"/>
@@ -86,12 +115,17 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B2A4A"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -120,7 +154,6 @@
       <bottom style="thin">
         <color rgb="FF1B2A4A"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -135,26 +168,28 @@
       <bottom style="thin">
         <color rgb="FFDDE3EC"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -451,16 +486,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -471,132 +506,132 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2">
+      <c r="A2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3">
+      <c r="A3" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4" t="n">
         <v>9.5</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+    <row r="6">
+      <c r="A6" s="5" t="n">
         <v>2024</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>2024</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" s="2"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="4"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10">
       <c r="A10" s="2"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="4"/>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11">
       <c r="A11" s="2"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="4"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="4"/>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12">
       <c r="A12" s="2"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="4"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="4"/>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13">
       <c r="A13" s="2"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="4"/>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14">
       <c r="A14" s="2"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="4"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15">
       <c r="A15" s="2"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="4"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="4"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16">
       <c r="A16" s="2"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="4"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="4"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17">
       <c r="A17" s="2"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="4"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18">
       <c r="A18" s="2"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -605,15 +640,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -621,51 +656,51 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2">
+      <c r="A2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="6" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3">
+      <c r="A3" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="6" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="6" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="6" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="6">
+      <c r="A6" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="6" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="6" t="n">
         <v>100</v>
       </c>
     </row>
@@ -676,15 +711,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,51 +727,51 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2">
+      <c r="A2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3">
+      <c r="A3" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="6">
+      <c r="A6" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -747,36 +782,57 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="52.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show general inputs first on the Data step and as the first sheet
Rename the Data step's "Data parameters" heading to "General inputs" and move it
to the top of the left column, above the losses preview. Create the general
inputs sheet first in make_example.R and reorder input.xlsx so it is the
leftmost tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="2265" yWindow="2265" windowWidth="28800" windowHeight="15345" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="2265" yWindow="2265" windowWidth="28800" windowHeight="15345" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
+    <sheet name="general inputs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="losses" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="exposure" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="inflation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="general inputs" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -115,17 +115,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -173,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -188,9 +183,6 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,13 +784,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rework the modelling threshold and guard the severity body
Three related changes to the severity/threshold modelling:

- Make the modelling threshold strict (losses are modelled above it, not at
  it) and fix the kink/point-mass that appeared when the splice sat on the
  threshold.

- Bring back the reporting threshold as a required general input (Excel
  template, reader, Data step display, docs) and default the modelling
  threshold to it, so the model starts where the data becomes reliable.

- Warn (non-blocking) when the splice is raised so the lognormal body is
  fitted on too few losses, nudging back to the single-Pareto default; the
  body stays an opt-in refinement.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,55 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="2265" yWindow="2265" windowWidth="28800" windowHeight="15345" firstSheet="0" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="general inputs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="losses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="exposure" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="inflation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="general inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="losses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="exposure" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="inflation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>year</t>
-  </si>
-  <si>
-    <t>loss</t>
-  </si>
-  <si>
-    <t>line_of_business</t>
-  </si>
-  <si>
-    <t>fire</t>
-  </si>
-  <si>
-    <t>exposure</t>
-  </si>
-  <si>
-    <t>inflation</t>
-  </si>
-  <si>
-    <t>key</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>reporting_threshold</t>
-  </si>
-  <si>
-    <t>valuation_year</t>
-  </si>
-  <si>
-    <t>2026</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -69,6 +35,15 @@
     <t xml:space="preserve">Required: the year losses are revalued to.</t>
   </si>
   <si>
+    <t xml:space="preserve">reporting_threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required: the loss size above which the data is complete.</t>
+  </si>
+  <si>
     <t xml:space="preserve">currency</t>
   </si>
   <si>
@@ -85,15 +60,34 @@
   </si>
   <si>
     <t xml:space="preserve">Optional: shown next to amounts (e.g. millions, thousands).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line_of_business</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exposure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inflation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+  <numFmts count="3">
+    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -168,35 +162,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -482,9 +463,9 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="52.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,135 +480,52 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B2" s="4" t="n">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B8" s="4" t="n">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="3"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="3"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="3"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="3"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="3"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -636,69 +534,212 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" s="6" t="n">
-        <v>100</v>
+      <c r="B2" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" s="6" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="B5" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" s="6" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="B7" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" s="6" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="B10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" s="6" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>100</v>
+      <c r="B15" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -707,69 +748,69 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>0</v>
+      <c r="B2" s="4" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>0</v>
+      <c r="B3" s="4" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" s="7" t="n">
-        <v>0</v>
+      <c r="B4" s="4" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>0</v>
+      <c r="B5" s="4" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>0</v>
+      <c r="B6" s="4" t="n">
+        <v>145</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>2026</v>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>0</v>
+      <c r="B7" s="4" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -778,57 +819,68 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="52.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>16</v>
+      <c r="A2" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>19</v>
+      <c r="A3" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>22</v>
+      <c r="A4" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0.035</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use the notes experience-pricing example losses in the template
Replace the demo losses in build_template_workbook with the seven losses
from the Reinsurance Analytics experience-pricing example (Figure 8):
2021: 12, 9.5; 2023: 18; 2024: 13, 7, 11; 2025: 14 (no losses in 2022).
Exposure, inflation and the general inputs are unchanged. Regenerate the
shipped input.xlsx to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -555,7 +555,7 @@
         <v>2021</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>18</v>
@@ -566,7 +566,7 @@
         <v>2021</v>
       </c>
       <c r="B3" s="4" t="n">
-        <v>8</v>
+        <v>9.5</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>18</v>
@@ -574,10 +574,10 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
@@ -585,10 +585,10 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>18</v>
@@ -596,10 +596,10 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
@@ -607,10 +607,10 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>18</v>
@@ -618,122 +618,12 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B8" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="C18" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add last complete experience year to the observation window
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -42,6 +42,15 @@
   </si>
   <si>
     <t xml:space="preserve">Required: the loss size above which the data is complete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_complete_year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional: the last year with complete loss data. Defaults to the latest loss year.</t>
   </si>
   <si>
     <t xml:space="preserve">currency</t>
@@ -523,6 +532,17 @@
         <v>14</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -541,13 +561,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2">
@@ -558,7 +578,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -569,7 +589,7 @@
         <v>9.5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -580,7 +600,7 @@
         <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -591,7 +611,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -602,7 +622,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -613,7 +633,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -624,7 +644,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -644,10 +664,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
@@ -715,10 +735,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2">

</xml_diff>